<commit_message>
feat(financials): record verified VA pay for July, update P&L to $6,222.44 loss
Real Airwallex payout confirmed: $105.00 USD, invoice #01 covering CS
support 2026-07-16 to 2026-07-31, settled 2026-08-01, rate $7.00/hour.
NOVA Cape Town had zero orders in this exact window (Sloane & Pearl had
97), so the full amount is attributable to Sloane & Pearl rather than
split pro-rata.

Updates the P&L, narrative, video script, and README to the corrected
90-day loss of $6,222.44 (was $6,117.44). Name-disclosure decision for
the CS contractor remains explicitly pending, per
disclosure/labor-attestation.md.
</commit_message>
<xml_diff>
--- a/financials/pnl-sloane-pearl.xlsx
+++ b/financials/pnl-sloane-pearl.xlsx
@@ -843,11 +843,13 @@
       </c>
       <c r="C15" s="20"/>
       <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
+      <c r="E15" s="20">
+        <v>105</v>
+      </c>
       <c r="F15" s="20"/>
       <c r="G15" s="21">
         <f>SUM(C15:F15)</f>
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="H15" s="18"/>
     </row>
@@ -1004,7 +1006,7 @@
       </c>
       <c r="E24" s="26">
         <f>E15+E16+E17+E19+E20+E21+E23</f>
-        <v>14221.27</v>
+        <v>14326.27</v>
       </c>
       <c r="F24" s="26">
         <f>F15+F16+F17+F19+F20+F21+F23</f>
@@ -1012,7 +1014,7 @@
       </c>
       <c r="G24" s="26">
         <f>G15+G16+G17+G19+G20+G21+G23</f>
-        <v>20096.62</v>
+        <v>20201.62</v>
       </c>
       <c r="H24" s="8"/>
     </row>
@@ -1041,7 +1043,7 @@
       </c>
       <c r="E26" s="32">
         <f>E11-E24</f>
-        <v>-2200.85</v>
+        <v>-2305.85</v>
       </c>
       <c r="F26" s="32">
         <f>F11-F24</f>
@@ -1049,7 +1051,7 @@
       </c>
       <c r="G26" s="32">
         <f>SUM(C26:F26)</f>
-        <v>-6117.44</v>
+        <v>-6222.44</v>
       </c>
       <c r="H26" s="7"/>
     </row>

</xml_diff>